<commit_message>
Added date validation engine.
</commit_message>
<xml_diff>
--- a/data/dashboard.xlsx
+++ b/data/dashboard.xlsx
@@ -24,12 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>invoice_id</t>
   </si>
   <si>
     <t>amount</t>
+  </si>
+  <si>
+    <t>sale_date</t>
   </si>
 </sst>
 </file>
@@ -88,13 +91,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -376,54 +384,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
     <col min="2" max="2" width="14.44140625" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1001</v>
       </c>
       <c r="B2" s="2">
         <v>1000</v>
       </c>
+      <c r="C2" s="4">
+        <v>46204</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1002</v>
       </c>
       <c r="B3" s="2">
         <v>2000</v>
       </c>
+      <c r="C3" s="5">
+        <v>46208</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1003</v>
       </c>
       <c r="B4" s="2">
         <v>3000</v>
       </c>
+      <c r="C4" s="4">
+        <v>46213</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1002</v>
       </c>
       <c r="B5" s="2">
         <v>2000</v>
+      </c>
+      <c r="C5" s="4">
+        <v>46218</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>